<commit_message>
ajout bouton détail métier
</commit_message>
<xml_diff>
--- a/public/modele_alimentation_pilotageh.xlsx
+++ b/public/modele_alimentation_pilotageh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\EMECI\COURS\M2PID 2\Lean Management\Dashboard\PilotageH_autonome\PilotageH_autonome\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{611CD23A-CF50-453C-B2CB-21ED46A60F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBD9581-2B07-4323-B9B5-BFF1E69EA2B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -512,7 +512,7 @@
       </c>
       <c r="F2" s="3">
         <f ca="1">RANDBETWEEN(DATE(2026,1,1),DATE(2026,12,31))</f>
-        <v>46141</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -533,7 +533,7 @@
       </c>
       <c r="F3" s="3">
         <f ca="1">RANDBETWEEN(DATE(2026,1,1),DATE(2026,12,31))</f>
-        <v>46138</v>
+        <v>46118</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -545,19 +545,19 @@
       </c>
       <c r="C4" s="1">
         <f ca="1">RANDBETWEEN(100,2500)</f>
-        <v>1826</v>
+        <v>1270</v>
       </c>
       <c r="D4" s="1">
         <f ca="1">RANDBETWEEN(100,E4)</f>
-        <v>816</v>
+        <v>299</v>
       </c>
       <c r="E4" s="1">
-        <f t="shared" ref="D4:E19" ca="1" si="0">RANDBETWEEN(100,2500)</f>
-        <v>2481</v>
+        <f t="shared" ref="E4:E19" ca="1" si="0">RANDBETWEEN(100,2500)</f>
+        <v>316</v>
       </c>
       <c r="F4" s="3">
         <f t="shared" ref="F4:F52" ca="1" si="1">RANDBETWEEN(DATE(2026,1,1),DATE(2026,12,31))</f>
-        <v>46258</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -569,19 +569,19 @@
       </c>
       <c r="C5" s="1">
         <f t="shared" ref="C5:C52" ca="1" si="2">RANDBETWEEN(100,2500)</f>
-        <v>837</v>
+        <v>428</v>
       </c>
       <c r="D5" s="1">
         <f t="shared" ref="D5:D52" ca="1" si="3">RANDBETWEEN(100,E5)</f>
-        <v>372</v>
+        <v>504</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>492</v>
+        <v>1668</v>
       </c>
       <c r="F5" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46081</v>
+        <v>46084</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -593,19 +593,19 @@
       </c>
       <c r="C6" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2149</v>
+        <v>2221</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>563</v>
+        <v>2168</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1719</v>
+        <v>2460</v>
       </c>
       <c r="F6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46215</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -617,19 +617,19 @@
       </c>
       <c r="C7" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>597</v>
+        <v>1857</v>
       </c>
       <c r="D7" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>240</v>
+        <v>212</v>
       </c>
       <c r="E7" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>433</v>
+        <v>243</v>
       </c>
       <c r="F7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46264</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -641,19 +641,19 @@
       </c>
       <c r="C8" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1162</v>
+        <v>1631</v>
       </c>
       <c r="D8" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>257</v>
+        <v>401</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>345</v>
+        <v>571</v>
       </c>
       <c r="F8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46096</v>
+        <v>46344</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -665,19 +665,19 @@
       </c>
       <c r="C9" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1889</v>
+        <v>1142</v>
       </c>
       <c r="D9" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>363</v>
+        <v>409</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2320</v>
+        <v>1608</v>
       </c>
       <c r="F9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46234</v>
+        <v>46202</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -689,19 +689,19 @@
       </c>
       <c r="C10" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>226</v>
+        <v>1756</v>
       </c>
       <c r="D10" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>896</v>
+        <v>135</v>
       </c>
       <c r="E10" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2439</v>
+        <v>163</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46032</v>
+        <v>46270</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -713,19 +713,19 @@
       </c>
       <c r="C11" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>352</v>
+        <v>752</v>
       </c>
       <c r="D11" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>629</v>
+        <v>1736</v>
       </c>
       <c r="E11" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>755</v>
+        <v>2442</v>
       </c>
       <c r="F11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46051</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -737,19 +737,19 @@
       </c>
       <c r="C12" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>900</v>
+        <v>602</v>
       </c>
       <c r="D12" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>726</v>
+        <v>478</v>
       </c>
       <c r="E12" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>970</v>
+        <v>1484</v>
       </c>
       <c r="F12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46048</v>
+        <v>46275</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -761,19 +761,19 @@
       </c>
       <c r="C13" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1636</v>
+        <v>653</v>
       </c>
       <c r="D13" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>225</v>
+        <v>108</v>
       </c>
       <c r="E13" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1881</v>
+        <v>158</v>
       </c>
       <c r="F13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46265</v>
+        <v>46379</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -785,19 +785,19 @@
       </c>
       <c r="C14" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1341</v>
+        <v>1713</v>
       </c>
       <c r="D14" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>823</v>
+        <v>1058</v>
       </c>
       <c r="E14" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>841</v>
+        <v>2310</v>
       </c>
       <c r="F14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46323</v>
+        <v>46183</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -809,19 +809,19 @@
       </c>
       <c r="C15" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1250</v>
+        <v>1942</v>
       </c>
       <c r="D15" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>119</v>
+        <v>713</v>
       </c>
       <c r="E15" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1758</v>
+        <v>1784</v>
       </c>
       <c r="F15" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46378</v>
+        <v>46382</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -833,19 +833,19 @@
       </c>
       <c r="C16" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>323</v>
+        <v>1519</v>
       </c>
       <c r="D16" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>121</v>
+        <v>499</v>
       </c>
       <c r="E16" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>321</v>
+        <v>2128</v>
       </c>
       <c r="F16" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46200</v>
+        <v>46024</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -857,19 +857,19 @@
       </c>
       <c r="C17" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>985</v>
+        <v>1359</v>
       </c>
       <c r="D17" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1367</v>
+        <v>248</v>
       </c>
       <c r="E17" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2000</v>
+        <v>535</v>
       </c>
       <c r="F17" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46234</v>
+        <v>46312</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -881,19 +881,19 @@
       </c>
       <c r="C18" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1994</v>
+        <v>564</v>
       </c>
       <c r="D18" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>215</v>
+        <v>560</v>
       </c>
       <c r="E18" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>323</v>
+        <v>963</v>
       </c>
       <c r="F18" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46151</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -905,19 +905,19 @@
       </c>
       <c r="C19" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>497</v>
+        <v>1317</v>
       </c>
       <c r="D19" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1796</v>
+        <v>927</v>
       </c>
       <c r="E19" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2118</v>
+        <v>1725</v>
       </c>
       <c r="F19" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46128</v>
+        <v>46111</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -929,19 +929,19 @@
       </c>
       <c r="C20" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1527</v>
+        <v>655</v>
       </c>
       <c r="D20" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>535</v>
+        <v>1833</v>
       </c>
       <c r="E20" s="1">
         <f t="shared" ref="E20:E52" ca="1" si="4">RANDBETWEEN(100,2500)</f>
-        <v>818</v>
+        <v>1952</v>
       </c>
       <c r="F20" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46237</v>
+        <v>46329</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -953,19 +953,19 @@
       </c>
       <c r="C21" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>365</v>
+        <v>386</v>
       </c>
       <c r="D21" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>171</v>
+        <v>556</v>
       </c>
       <c r="E21" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>921</v>
+        <v>749</v>
       </c>
       <c r="F21" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46080</v>
+        <v>46127</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -977,19 +977,19 @@
       </c>
       <c r="C22" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>724</v>
+        <v>2092</v>
       </c>
       <c r="D22" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1081</v>
+        <v>1060</v>
       </c>
       <c r="E22" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1219</v>
+        <v>1341</v>
       </c>
       <c r="F22" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46077</v>
+        <v>46106</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -1001,19 +1001,19 @@
       </c>
       <c r="C23" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>332</v>
+        <v>306</v>
       </c>
       <c r="D23" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1026</v>
+        <v>2189</v>
       </c>
       <c r="E23" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1542</v>
+        <v>2246</v>
       </c>
       <c r="F23" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46139</v>
+        <v>46160</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1025,19 +1025,19 @@
       </c>
       <c r="C24" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1322</v>
+        <v>1521</v>
       </c>
       <c r="D24" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>585</v>
+        <v>551</v>
       </c>
       <c r="E24" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2266</v>
+        <v>749</v>
       </c>
       <c r="F24" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46221</v>
+        <v>46109</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -1049,19 +1049,19 @@
       </c>
       <c r="C25" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1842</v>
+        <v>717</v>
       </c>
       <c r="D25" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>468</v>
+        <v>454</v>
       </c>
       <c r="E25" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1656</v>
+        <v>707</v>
       </c>
       <c r="F25" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46370</v>
+        <v>46198</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="C26" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2266</v>
+        <v>2132</v>
       </c>
       <c r="D26" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>356</v>
+        <v>1512</v>
       </c>
       <c r="E26" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1996</v>
+        <v>2036</v>
       </c>
       <c r="F26" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46291</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -1097,19 +1097,19 @@
       </c>
       <c r="C27" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2208</v>
+        <v>1581</v>
       </c>
       <c r="D27" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>130</v>
+        <v>420</v>
       </c>
       <c r="E27" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>133</v>
+        <v>669</v>
       </c>
       <c r="F27" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46154</v>
+        <v>46139</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -1121,19 +1121,19 @@
       </c>
       <c r="C28" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>591</v>
+        <v>2003</v>
       </c>
       <c r="D28" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1304</v>
+        <v>1301</v>
       </c>
       <c r="E28" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1472</v>
+        <v>2175</v>
       </c>
       <c r="F28" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46372</v>
+        <v>46170</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -1145,19 +1145,19 @@
       </c>
       <c r="C29" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>450</v>
+        <v>1523</v>
       </c>
       <c r="D29" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1627</v>
+        <v>225</v>
       </c>
       <c r="E29" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2324</v>
+        <v>1363</v>
       </c>
       <c r="F29" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46228</v>
+        <v>46026</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -1169,19 +1169,19 @@
       </c>
       <c r="C30" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>692</v>
+        <v>154</v>
       </c>
       <c r="D30" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>593</v>
+        <v>1979</v>
       </c>
       <c r="E30" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>802</v>
+        <v>1993</v>
       </c>
       <c r="F30" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46204</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -1193,19 +1193,19 @@
       </c>
       <c r="C31" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1421</v>
+        <v>228</v>
       </c>
       <c r="D31" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1436</v>
+        <v>113</v>
       </c>
       <c r="E31" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1837</v>
+        <v>148</v>
       </c>
       <c r="F31" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46151</v>
+        <v>46360</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
@@ -1217,19 +1217,19 @@
       </c>
       <c r="C32" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1261</v>
+        <v>981</v>
       </c>
       <c r="D32" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>197</v>
+        <v>170</v>
       </c>
       <c r="E32" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>637</v>
+        <v>204</v>
       </c>
       <c r="F32" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46172</v>
+        <v>46249</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
@@ -1241,19 +1241,19 @@
       </c>
       <c r="C33" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>406</v>
+        <v>2085</v>
       </c>
       <c r="D33" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>540</v>
+        <v>124</v>
       </c>
       <c r="E33" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>973</v>
+        <v>648</v>
       </c>
       <c r="F33" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46144</v>
+        <v>46136</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -1265,19 +1265,19 @@
       </c>
       <c r="C34" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1826</v>
+        <v>1584</v>
       </c>
       <c r="D34" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>884</v>
+        <v>104</v>
       </c>
       <c r="E34" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1043</v>
+        <v>135</v>
       </c>
       <c r="F34" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46300</v>
+        <v>46322</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
@@ -1289,19 +1289,19 @@
       </c>
       <c r="C35" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2017</v>
+        <v>471</v>
       </c>
       <c r="D35" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>170</v>
+        <v>490</v>
       </c>
       <c r="E35" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1848</v>
+        <v>1642</v>
       </c>
       <c r="F35" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46312</v>
+        <v>46351</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
@@ -1313,19 +1313,19 @@
       </c>
       <c r="C36" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1001</v>
+        <v>970</v>
       </c>
       <c r="D36" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1555</v>
+        <v>1207</v>
       </c>
       <c r="E36" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1757</v>
+        <v>2263</v>
       </c>
       <c r="F36" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46063</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -1337,19 +1337,19 @@
       </c>
       <c r="C37" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1347</v>
+        <v>2453</v>
       </c>
       <c r="D37" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>913</v>
+        <v>533</v>
       </c>
       <c r="E37" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>970</v>
+        <v>1280</v>
       </c>
       <c r="F37" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46175</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -1361,19 +1361,19 @@
       </c>
       <c r="C38" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>862</v>
+        <v>411</v>
       </c>
       <c r="D38" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>167</v>
+        <v>118</v>
       </c>
       <c r="E38" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1232</v>
+        <v>284</v>
       </c>
       <c r="F38" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46030</v>
+        <v>46218</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -1385,19 +1385,19 @@
       </c>
       <c r="C39" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2179</v>
+        <v>120</v>
       </c>
       <c r="D39" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>770</v>
+        <v>1311</v>
       </c>
       <c r="E39" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1926</v>
+        <v>2134</v>
       </c>
       <c r="F39" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46037</v>
+        <v>46188</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -1409,19 +1409,19 @@
       </c>
       <c r="C40" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1756</v>
+        <v>1578</v>
       </c>
       <c r="D40" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1074</v>
+        <v>1546</v>
       </c>
       <c r="E40" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2278</v>
+        <v>1564</v>
       </c>
       <c r="F40" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46163</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -1433,19 +1433,19 @@
       </c>
       <c r="C41" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1646</v>
+        <v>810</v>
       </c>
       <c r="D41" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>506</v>
+        <v>1059</v>
       </c>
       <c r="E41" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2179</v>
+        <v>1487</v>
       </c>
       <c r="F41" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46334</v>
+        <v>46076</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -1457,19 +1457,19 @@
       </c>
       <c r="C42" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1618</v>
+        <v>1069</v>
       </c>
       <c r="D42" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>207</v>
+        <v>129</v>
       </c>
       <c r="E42" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>475</v>
+        <v>168</v>
       </c>
       <c r="F42" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46361</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1481,19 +1481,19 @@
       </c>
       <c r="C43" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2155</v>
+        <v>817</v>
       </c>
       <c r="D43" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>453</v>
+        <v>444</v>
       </c>
       <c r="E43" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>654</v>
+        <v>851</v>
       </c>
       <c r="F43" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46361</v>
+        <v>46343</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -1505,19 +1505,19 @@
       </c>
       <c r="C44" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2314</v>
+        <v>829</v>
       </c>
       <c r="D44" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1444</v>
+        <v>1343</v>
       </c>
       <c r="E44" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2474</v>
+        <v>1948</v>
       </c>
       <c r="F44" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46371</v>
+        <v>46356</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -1529,19 +1529,19 @@
       </c>
       <c r="C45" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2103</v>
+        <v>994</v>
       </c>
       <c r="D45" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E45" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1659</v>
+        <v>979</v>
       </c>
       <c r="F45" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46227</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1553,19 +1553,19 @@
       </c>
       <c r="C46" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>656</v>
+        <v>516</v>
       </c>
       <c r="D46" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1613</v>
+        <v>446</v>
       </c>
       <c r="E46" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2283</v>
+        <v>1516</v>
       </c>
       <c r="F46" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46302</v>
+        <v>46067</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -1577,19 +1577,19 @@
       </c>
       <c r="C47" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2436</v>
+        <v>1764</v>
       </c>
       <c r="D47" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1580</v>
+        <v>1293</v>
       </c>
       <c r="E47" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2428</v>
+        <v>2044</v>
       </c>
       <c r="F47" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46089</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -1601,19 +1601,19 @@
       </c>
       <c r="C48" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>540</v>
+        <v>1756</v>
       </c>
       <c r="D48" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>536</v>
+        <v>511</v>
       </c>
       <c r="E48" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1563</v>
+        <v>1815</v>
       </c>
       <c r="F48" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46360</v>
+        <v>46079</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -1625,19 +1625,19 @@
       </c>
       <c r="C49" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>310</v>
+        <v>1021</v>
       </c>
       <c r="D49" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="E49" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>780</v>
+        <v>543</v>
       </c>
       <c r="F49" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46362</v>
+        <v>46080</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -1649,19 +1649,19 @@
       </c>
       <c r="C50" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1785</v>
+        <v>200</v>
       </c>
       <c r="D50" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>509</v>
+        <v>139</v>
       </c>
       <c r="E50" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1332</v>
+        <v>707</v>
       </c>
       <c r="F50" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46266</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -1673,19 +1673,19 @@
       </c>
       <c r="C51" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1178</v>
+        <v>1032</v>
       </c>
       <c r="D51" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>619</v>
+        <v>1039</v>
       </c>
       <c r="E51" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1500</v>
+        <v>2261</v>
       </c>
       <c r="F51" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46196</v>
+        <v>46263</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -1697,19 +1697,19 @@
       </c>
       <c r="C52" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2167</v>
+        <v>2346</v>
       </c>
       <c r="D52" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>306</v>
+        <v>459</v>
       </c>
       <c r="E52" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1455</v>
+        <v>656</v>
       </c>
       <c r="F52" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46143</v>
+        <v>46305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: synchronisation dynamique des métiers depuis Excel
</commit_message>
<xml_diff>
--- a/public/modele_alimentation_pilotageh.xlsx
+++ b/public/modele_alimentation_pilotageh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\EMECI\COURS\M2PID 2\Lean Management\Dashboard\PilotageH_autonome\PilotageH_autonome\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBD9581-2B07-4323-B9B5-BFF1E69EA2B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C0EA33E-7A68-4B67-BEF8-21CED1011929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -104,7 +104,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,6 +116,12 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -512,7 +518,7 @@
       </c>
       <c r="F2" s="3">
         <f ca="1">RANDBETWEEN(DATE(2026,1,1),DATE(2026,12,31))</f>
-        <v>46197</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -533,7 +539,7 @@
       </c>
       <c r="F3" s="3">
         <f ca="1">RANDBETWEEN(DATE(2026,1,1),DATE(2026,12,31))</f>
-        <v>46118</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -545,19 +551,19 @@
       </c>
       <c r="C4" s="1">
         <f ca="1">RANDBETWEEN(100,2500)</f>
-        <v>1270</v>
+        <v>484</v>
       </c>
       <c r="D4" s="1">
         <f ca="1">RANDBETWEEN(100,E4)</f>
-        <v>299</v>
+        <v>675</v>
       </c>
       <c r="E4" s="1">
         <f t="shared" ref="E4:E19" ca="1" si="0">RANDBETWEEN(100,2500)</f>
-        <v>316</v>
+        <v>1359</v>
       </c>
       <c r="F4" s="3">
         <f t="shared" ref="F4:F52" ca="1" si="1">RANDBETWEEN(DATE(2026,1,1),DATE(2026,12,31))</f>
-        <v>46172</v>
+        <v>46340</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -569,19 +575,19 @@
       </c>
       <c r="C5" s="1">
         <f t="shared" ref="C5:C52" ca="1" si="2">RANDBETWEEN(100,2500)</f>
-        <v>428</v>
+        <v>524</v>
       </c>
       <c r="D5" s="1">
         <f t="shared" ref="D5:D52" ca="1" si="3">RANDBETWEEN(100,E5)</f>
-        <v>504</v>
+        <v>565</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1668</v>
+        <v>586</v>
       </c>
       <c r="F5" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46084</v>
+        <v>46363</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -593,19 +599,19 @@
       </c>
       <c r="C6" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2221</v>
+        <v>2316</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>2168</v>
+        <v>196</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2460</v>
+        <v>786</v>
       </c>
       <c r="F6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46236</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -617,19 +623,19 @@
       </c>
       <c r="C7" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1857</v>
+        <v>338</v>
       </c>
       <c r="D7" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>212</v>
+        <v>1406</v>
       </c>
       <c r="E7" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>243</v>
+        <v>2096</v>
       </c>
       <c r="F7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46252</v>
+        <v>46342</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -641,19 +647,19 @@
       </c>
       <c r="C8" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1631</v>
+        <v>548</v>
       </c>
       <c r="D8" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>401</v>
+        <v>851</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>571</v>
+        <v>1445</v>
       </c>
       <c r="F8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46344</v>
+        <v>46041</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -665,19 +671,19 @@
       </c>
       <c r="C9" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1142</v>
+        <v>1319</v>
       </c>
       <c r="D9" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>409</v>
+        <v>356</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1608</v>
+        <v>1315</v>
       </c>
       <c r="F9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46202</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -689,19 +695,19 @@
       </c>
       <c r="C10" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1756</v>
+        <v>131</v>
       </c>
       <c r="D10" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>135</v>
+        <v>343</v>
       </c>
       <c r="E10" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>163</v>
+        <v>369</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46270</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -713,19 +719,19 @@
       </c>
       <c r="C11" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>752</v>
+        <v>473</v>
       </c>
       <c r="D11" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1736</v>
+        <v>2201</v>
       </c>
       <c r="E11" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2442</v>
+        <v>2282</v>
       </c>
       <c r="F11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46274</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -737,19 +743,19 @@
       </c>
       <c r="C12" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>602</v>
+        <v>2382</v>
       </c>
       <c r="D12" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>478</v>
+        <v>141</v>
       </c>
       <c r="E12" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1484</v>
+        <v>390</v>
       </c>
       <c r="F12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46275</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -761,19 +767,19 @@
       </c>
       <c r="C13" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>653</v>
+        <v>1885</v>
       </c>
       <c r="D13" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="E13" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>158</v>
+        <v>2351</v>
       </c>
       <c r="F13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46379</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -785,19 +791,19 @@
       </c>
       <c r="C14" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1713</v>
+        <v>1458</v>
       </c>
       <c r="D14" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1058</v>
+        <v>163</v>
       </c>
       <c r="E14" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2310</v>
+        <v>243</v>
       </c>
       <c r="F14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46183</v>
+        <v>46242</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -809,19 +815,19 @@
       </c>
       <c r="C15" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1942</v>
+        <v>2060</v>
       </c>
       <c r="D15" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>713</v>
+        <v>648</v>
       </c>
       <c r="E15" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1784</v>
+        <v>1567</v>
       </c>
       <c r="F15" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46382</v>
+        <v>46350</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -833,19 +839,19 @@
       </c>
       <c r="C16" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1519</v>
+        <v>2289</v>
       </c>
       <c r="D16" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>499</v>
+        <v>1560</v>
       </c>
       <c r="E16" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2128</v>
+        <v>2255</v>
       </c>
       <c r="F16" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46024</v>
+        <v>46353</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -857,19 +863,19 @@
       </c>
       <c r="C17" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1359</v>
+        <v>1215</v>
       </c>
       <c r="D17" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>248</v>
+        <v>342</v>
       </c>
       <c r="E17" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>535</v>
+        <v>1602</v>
       </c>
       <c r="F17" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46312</v>
+        <v>46074</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -881,19 +887,19 @@
       </c>
       <c r="C18" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>564</v>
+        <v>1264</v>
       </c>
       <c r="D18" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>560</v>
+        <v>351</v>
       </c>
       <c r="E18" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>963</v>
+        <v>1239</v>
       </c>
       <c r="F18" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46293</v>
+        <v>46249</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -905,19 +911,19 @@
       </c>
       <c r="C19" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1317</v>
+        <v>1219</v>
       </c>
       <c r="D19" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>927</v>
+        <v>407</v>
       </c>
       <c r="E19" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1725</v>
+        <v>506</v>
       </c>
       <c r="F19" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46111</v>
+        <v>46263</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -929,19 +935,19 @@
       </c>
       <c r="C20" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>655</v>
+        <v>1156</v>
       </c>
       <c r="D20" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1833</v>
+        <v>836</v>
       </c>
       <c r="E20" s="1">
         <f t="shared" ref="E20:E52" ca="1" si="4">RANDBETWEEN(100,2500)</f>
-        <v>1952</v>
+        <v>1096</v>
       </c>
       <c r="F20" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46329</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -953,19 +959,19 @@
       </c>
       <c r="C21" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>386</v>
+        <v>126</v>
       </c>
       <c r="D21" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>556</v>
+        <v>120</v>
       </c>
       <c r="E21" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>749</v>
+        <v>125</v>
       </c>
       <c r="F21" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46127</v>
+        <v>46257</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -977,19 +983,19 @@
       </c>
       <c r="C22" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2092</v>
+        <v>581</v>
       </c>
       <c r="D22" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1060</v>
+        <v>300</v>
       </c>
       <c r="E22" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1341</v>
+        <v>1076</v>
       </c>
       <c r="F22" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46106</v>
+        <v>46118</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -1001,19 +1007,19 @@
       </c>
       <c r="C23" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>306</v>
+        <v>1595</v>
       </c>
       <c r="D23" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>2189</v>
+        <v>1692</v>
       </c>
       <c r="E23" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2246</v>
+        <v>2094</v>
       </c>
       <c r="F23" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46160</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1025,19 +1031,19 @@
       </c>
       <c r="C24" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1521</v>
+        <v>399</v>
       </c>
       <c r="D24" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>551</v>
+        <v>239</v>
       </c>
       <c r="E24" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>749</v>
+        <v>279</v>
       </c>
       <c r="F24" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46109</v>
+        <v>46353</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -1049,19 +1055,19 @@
       </c>
       <c r="C25" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>717</v>
+        <v>1702</v>
       </c>
       <c r="D25" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>454</v>
+        <v>167</v>
       </c>
       <c r="E25" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>707</v>
+        <v>281</v>
       </c>
       <c r="F25" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46198</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -1073,19 +1079,19 @@
       </c>
       <c r="C26" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2132</v>
+        <v>1741</v>
       </c>
       <c r="D26" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1512</v>
+        <v>392</v>
       </c>
       <c r="E26" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2036</v>
+        <v>1761</v>
       </c>
       <c r="F26" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46108</v>
+        <v>46269</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -1097,19 +1103,19 @@
       </c>
       <c r="C27" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1581</v>
+        <v>967</v>
       </c>
       <c r="D27" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>420</v>
+        <v>308</v>
       </c>
       <c r="E27" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>669</v>
+        <v>630</v>
       </c>
       <c r="F27" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46139</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -1121,19 +1127,19 @@
       </c>
       <c r="C28" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2003</v>
+        <v>1488</v>
       </c>
       <c r="D28" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1301</v>
+        <v>973</v>
       </c>
       <c r="E28" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2175</v>
+        <v>2240</v>
       </c>
       <c r="F28" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46170</v>
+        <v>46190</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -1145,19 +1151,19 @@
       </c>
       <c r="C29" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1523</v>
+        <v>2370</v>
       </c>
       <c r="D29" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>225</v>
+        <v>274</v>
       </c>
       <c r="E29" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1363</v>
+        <v>1061</v>
       </c>
       <c r="F29" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46026</v>
+        <v>46063</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -1169,19 +1175,19 @@
       </c>
       <c r="C30" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D30" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1979</v>
+        <v>1190</v>
       </c>
       <c r="E30" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1993</v>
+        <v>1912</v>
       </c>
       <c r="F30" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46295</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -1193,19 +1199,19 @@
       </c>
       <c r="C31" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>228</v>
+        <v>370</v>
       </c>
       <c r="D31" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>113</v>
+        <v>1458</v>
       </c>
       <c r="E31" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>148</v>
+        <v>2399</v>
       </c>
       <c r="F31" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46360</v>
+        <v>46066</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
@@ -1217,19 +1223,19 @@
       </c>
       <c r="C32" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>981</v>
+        <v>1234</v>
       </c>
       <c r="D32" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="E32" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>204</v>
+        <v>1156</v>
       </c>
       <c r="F32" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46249</v>
+        <v>46365</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
@@ -1241,19 +1247,19 @@
       </c>
       <c r="C33" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2085</v>
+        <v>1865</v>
       </c>
       <c r="D33" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>124</v>
+        <v>346</v>
       </c>
       <c r="E33" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>648</v>
+        <v>400</v>
       </c>
       <c r="F33" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46136</v>
+        <v>46114</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -1265,19 +1271,19 @@
       </c>
       <c r="C34" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1584</v>
+        <v>1786</v>
       </c>
       <c r="D34" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>104</v>
+        <v>460</v>
       </c>
       <c r="E34" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>135</v>
+        <v>1429</v>
       </c>
       <c r="F34" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46322</v>
+        <v>46035</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
@@ -1289,19 +1295,19 @@
       </c>
       <c r="C35" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>471</v>
+        <v>315</v>
       </c>
       <c r="D35" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>490</v>
+        <v>156</v>
       </c>
       <c r="E35" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1642</v>
+        <v>254</v>
       </c>
       <c r="F35" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46351</v>
+        <v>46387</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
@@ -1313,19 +1319,19 @@
       </c>
       <c r="C36" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>970</v>
+        <v>554</v>
       </c>
       <c r="D36" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1207</v>
+        <v>713</v>
       </c>
       <c r="E36" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2263</v>
+        <v>1562</v>
       </c>
       <c r="F36" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46310</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -1337,19 +1343,19 @@
       </c>
       <c r="C37" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2453</v>
+        <v>1383</v>
       </c>
       <c r="D37" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>533</v>
+        <v>1754</v>
       </c>
       <c r="E37" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1280</v>
+        <v>2152</v>
       </c>
       <c r="F37" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46234</v>
+        <v>46046</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -1361,19 +1367,19 @@
       </c>
       <c r="C38" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>411</v>
+        <v>665</v>
       </c>
       <c r="D38" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>118</v>
+        <v>468</v>
       </c>
       <c r="E38" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>284</v>
+        <v>576</v>
       </c>
       <c r="F38" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46218</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -1385,19 +1391,19 @@
       </c>
       <c r="C39" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>120</v>
+        <v>165</v>
       </c>
       <c r="D39" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1311</v>
+        <v>383</v>
       </c>
       <c r="E39" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2134</v>
+        <v>1364</v>
       </c>
       <c r="F39" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46188</v>
+        <v>46083</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -1409,19 +1415,19 @@
       </c>
       <c r="C40" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1578</v>
+        <v>1610</v>
       </c>
       <c r="D40" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1546</v>
+        <v>239</v>
       </c>
       <c r="E40" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1564</v>
+        <v>2328</v>
       </c>
       <c r="F40" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46280</v>
+        <v>46269</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -1433,19 +1439,19 @@
       </c>
       <c r="C41" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>810</v>
+        <v>341</v>
       </c>
       <c r="D41" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1059</v>
+        <v>243</v>
       </c>
       <c r="E41" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1487</v>
+        <v>261</v>
       </c>
       <c r="F41" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46076</v>
+        <v>46181</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -1457,19 +1463,19 @@
       </c>
       <c r="C42" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1069</v>
+        <v>1437</v>
       </c>
       <c r="D42" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>129</v>
+        <v>404</v>
       </c>
       <c r="E42" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>168</v>
+        <v>955</v>
       </c>
       <c r="F42" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46321</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1481,19 +1487,19 @@
       </c>
       <c r="C43" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>817</v>
+        <v>1260</v>
       </c>
       <c r="D43" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>444</v>
+        <v>754</v>
       </c>
       <c r="E43" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>851</v>
+        <v>1208</v>
       </c>
       <c r="F43" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46343</v>
+        <v>46384</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -1505,19 +1511,19 @@
       </c>
       <c r="C44" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>829</v>
+        <v>1408</v>
       </c>
       <c r="D44" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1343</v>
+        <v>638</v>
       </c>
       <c r="E44" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1948</v>
+        <v>866</v>
       </c>
       <c r="F44" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46356</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -1529,19 +1535,19 @@
       </c>
       <c r="C45" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>994</v>
+        <v>1166</v>
       </c>
       <c r="D45" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>116</v>
+        <v>207</v>
       </c>
       <c r="E45" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>979</v>
+        <v>223</v>
       </c>
       <c r="F45" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46230</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1553,19 +1559,19 @@
       </c>
       <c r="C46" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>516</v>
+        <v>2095</v>
       </c>
       <c r="D46" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>446</v>
+        <v>568</v>
       </c>
       <c r="E46" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1516</v>
+        <v>652</v>
       </c>
       <c r="F46" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46067</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -1577,19 +1583,19 @@
       </c>
       <c r="C47" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1764</v>
+        <v>910</v>
       </c>
       <c r="D47" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1293</v>
+        <v>315</v>
       </c>
       <c r="E47" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2044</v>
+        <v>578</v>
       </c>
       <c r="F47" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46161</v>
+        <v>46024</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -1601,19 +1607,19 @@
       </c>
       <c r="C48" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1756</v>
+        <v>707</v>
       </c>
       <c r="D48" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>511</v>
+        <v>116</v>
       </c>
       <c r="E48" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1815</v>
+        <v>149</v>
       </c>
       <c r="F48" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46079</v>
+        <v>46208</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -1625,19 +1631,19 @@
       </c>
       <c r="C49" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1021</v>
+        <v>1597</v>
       </c>
       <c r="D49" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>286</v>
+        <v>1466</v>
       </c>
       <c r="E49" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>543</v>
+        <v>2254</v>
       </c>
       <c r="F49" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46080</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -1649,19 +1655,19 @@
       </c>
       <c r="C50" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>200</v>
+        <v>2448</v>
       </c>
       <c r="D50" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>139</v>
+        <v>1078</v>
       </c>
       <c r="E50" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>707</v>
+        <v>2323</v>
       </c>
       <c r="F50" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46227</v>
+        <v>46243</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -1673,19 +1679,19 @@
       </c>
       <c r="C51" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1032</v>
+        <v>2234</v>
       </c>
       <c r="D51" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1039</v>
+        <v>1069</v>
       </c>
       <c r="E51" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2261</v>
+        <v>1155</v>
       </c>
       <c r="F51" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46263</v>
+        <v>46193</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -1697,22 +1703,23 @@
       </c>
       <c r="C52" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2346</v>
+        <v>151</v>
       </c>
       <c r="D52" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>459</v>
+        <v>708</v>
       </c>
       <c r="E52" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>656</v>
+        <v>1111</v>
       </c>
       <c r="F52" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46305</v>
+        <v>46336</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Amélioration affichage histogrammes métiers
</commit_message>
<xml_diff>
--- a/public/modele_alimentation_pilotageh.xlsx
+++ b/public/modele_alimentation_pilotageh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\EMECI\COURS\M2PID 2\Lean Management\Dashboard\PilotageH_autonome\PilotageH_autonome\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C0EA33E-7A68-4B67-BEF8-21CED1011929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058F5E44-DB62-4810-9B35-6B92025AE483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -508,17 +508,17 @@
         <v>6</v>
       </c>
       <c r="C2" s="1">
+        <v>100</v>
+      </c>
+      <c r="D2" s="1">
         <v>120</v>
       </c>
-      <c r="D2" s="1">
-        <v>60</v>
-      </c>
       <c r="E2" s="1">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F2" s="3">
         <f ca="1">RANDBETWEEN(DATE(2026,1,1),DATE(2026,12,31))</f>
-        <v>46230</v>
+        <v>46079</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -539,7 +539,7 @@
       </c>
       <c r="F3" s="3">
         <f ca="1">RANDBETWEEN(DATE(2026,1,1),DATE(2026,12,31))</f>
-        <v>46145</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -551,19 +551,19 @@
       </c>
       <c r="C4" s="1">
         <f ca="1">RANDBETWEEN(100,2500)</f>
-        <v>484</v>
+        <v>1479</v>
       </c>
       <c r="D4" s="1">
         <f ca="1">RANDBETWEEN(100,E4)</f>
-        <v>675</v>
+        <v>734</v>
       </c>
       <c r="E4" s="1">
         <f t="shared" ref="E4:E19" ca="1" si="0">RANDBETWEEN(100,2500)</f>
-        <v>1359</v>
+        <v>2177</v>
       </c>
       <c r="F4" s="3">
         <f t="shared" ref="F4:F52" ca="1" si="1">RANDBETWEEN(DATE(2026,1,1),DATE(2026,12,31))</f>
-        <v>46340</v>
+        <v>46371</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -575,19 +575,19 @@
       </c>
       <c r="C5" s="1">
         <f t="shared" ref="C5:C52" ca="1" si="2">RANDBETWEEN(100,2500)</f>
-        <v>524</v>
+        <v>1222</v>
       </c>
       <c r="D5" s="1">
         <f t="shared" ref="D5:D52" ca="1" si="3">RANDBETWEEN(100,E5)</f>
-        <v>565</v>
+        <v>106</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>586</v>
+        <v>124</v>
       </c>
       <c r="F5" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46363</v>
+        <v>46087</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -599,19 +599,19 @@
       </c>
       <c r="C6" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2316</v>
+        <v>1321</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>196</v>
+        <v>1362</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>786</v>
+        <v>1716</v>
       </c>
       <c r="F6" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46208</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -623,19 +623,19 @@
       </c>
       <c r="C7" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>338</v>
+        <v>290</v>
       </c>
       <c r="D7" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1406</v>
+        <v>520</v>
       </c>
       <c r="E7" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2096</v>
+        <v>724</v>
       </c>
       <c r="F7" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46342</v>
+        <v>46075</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -647,19 +647,19 @@
       </c>
       <c r="C8" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>548</v>
+        <v>1550</v>
       </c>
       <c r="D8" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>851</v>
+        <v>1483</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1445</v>
+        <v>2072</v>
       </c>
       <c r="F8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46041</v>
+        <v>46343</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -671,19 +671,19 @@
       </c>
       <c r="C9" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1319</v>
+        <v>1022</v>
       </c>
       <c r="D9" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>356</v>
+        <v>104</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1315</v>
+        <v>673</v>
       </c>
       <c r="F9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46279</v>
+        <v>46370</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -695,19 +695,19 @@
       </c>
       <c r="C10" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>131</v>
+        <v>1346</v>
       </c>
       <c r="D10" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>343</v>
+        <v>489</v>
       </c>
       <c r="E10" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>369</v>
+        <v>561</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46231</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -719,19 +719,19 @@
       </c>
       <c r="C11" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>473</v>
+        <v>1843</v>
       </c>
       <c r="D11" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>2201</v>
+        <v>1821</v>
       </c>
       <c r="E11" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2282</v>
+        <v>1998</v>
       </c>
       <c r="F11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46128</v>
+        <v>46264</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -743,19 +743,19 @@
       </c>
       <c r="C12" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2382</v>
+        <v>2046</v>
       </c>
       <c r="D12" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>141</v>
+        <v>933</v>
       </c>
       <c r="E12" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>390</v>
+        <v>1325</v>
       </c>
       <c r="F12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46213</v>
+        <v>46097</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -767,19 +767,19 @@
       </c>
       <c r="C13" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1885</v>
+        <v>983</v>
       </c>
       <c r="D13" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="E13" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2351</v>
+        <v>357</v>
       </c>
       <c r="F13" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46217</v>
+        <v>46115</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -791,19 +791,19 @@
       </c>
       <c r="C14" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1458</v>
+        <v>1966</v>
       </c>
       <c r="D14" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>163</v>
+        <v>242</v>
       </c>
       <c r="E14" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>243</v>
+        <v>539</v>
       </c>
       <c r="F14" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46242</v>
+        <v>46180</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -815,19 +815,19 @@
       </c>
       <c r="C15" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2060</v>
+        <v>954</v>
       </c>
       <c r="D15" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>648</v>
+        <v>552</v>
       </c>
       <c r="E15" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1567</v>
+        <v>557</v>
       </c>
       <c r="F15" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46350</v>
+        <v>46030</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -839,19 +839,19 @@
       </c>
       <c r="C16" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2289</v>
+        <v>167</v>
       </c>
       <c r="D16" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1560</v>
+        <v>269</v>
       </c>
       <c r="E16" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>2255</v>
+        <v>685</v>
       </c>
       <c r="F16" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46353</v>
+        <v>46064</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -863,19 +863,19 @@
       </c>
       <c r="C17" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1215</v>
+        <v>1883</v>
       </c>
       <c r="D17" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>342</v>
+        <v>1164</v>
       </c>
       <c r="E17" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1602</v>
+        <v>2360</v>
       </c>
       <c r="F17" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46074</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -887,19 +887,19 @@
       </c>
       <c r="C18" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1264</v>
+        <v>2197</v>
       </c>
       <c r="D18" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>351</v>
+        <v>158</v>
       </c>
       <c r="E18" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>1239</v>
+        <v>207</v>
       </c>
       <c r="F18" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46249</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -911,19 +911,19 @@
       </c>
       <c r="C19" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1219</v>
+        <v>642</v>
       </c>
       <c r="D19" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>407</v>
+        <v>101</v>
       </c>
       <c r="E19" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>506</v>
+        <v>122</v>
       </c>
       <c r="F19" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46263</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -935,19 +935,19 @@
       </c>
       <c r="C20" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1156</v>
+        <v>1852</v>
       </c>
       <c r="D20" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>836</v>
+        <v>2206</v>
       </c>
       <c r="E20" s="1">
         <f t="shared" ref="E20:E52" ca="1" si="4">RANDBETWEEN(100,2500)</f>
-        <v>1096</v>
+        <v>2482</v>
       </c>
       <c r="F20" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46201</v>
+        <v>46353</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -959,19 +959,19 @@
       </c>
       <c r="C21" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>126</v>
+        <v>562</v>
       </c>
       <c r="D21" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>120</v>
+        <v>191</v>
       </c>
       <c r="E21" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>125</v>
+        <v>691</v>
       </c>
       <c r="F21" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46257</v>
+        <v>46099</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -983,19 +983,19 @@
       </c>
       <c r="C22" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>581</v>
+        <v>973</v>
       </c>
       <c r="D22" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>300</v>
+        <v>189</v>
       </c>
       <c r="E22" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1076</v>
+        <v>1224</v>
       </c>
       <c r="F22" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46118</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -1007,19 +1007,19 @@
       </c>
       <c r="C23" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1595</v>
+        <v>1350</v>
       </c>
       <c r="D23" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1692</v>
+        <v>1309</v>
       </c>
       <c r="E23" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2094</v>
+        <v>1534</v>
       </c>
       <c r="F23" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46174</v>
+        <v>46172</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1031,19 +1031,19 @@
       </c>
       <c r="C24" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>399</v>
+        <v>454</v>
       </c>
       <c r="D24" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>239</v>
+        <v>1298</v>
       </c>
       <c r="E24" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>279</v>
+        <v>1507</v>
       </c>
       <c r="F24" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46353</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -1055,19 +1055,19 @@
       </c>
       <c r="C25" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1702</v>
+        <v>2328</v>
       </c>
       <c r="D25" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>167</v>
+        <v>662</v>
       </c>
       <c r="E25" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>281</v>
+        <v>1567</v>
       </c>
       <c r="F25" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46219</v>
+        <v>46379</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -1079,19 +1079,19 @@
       </c>
       <c r="C26" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1741</v>
+        <v>773</v>
       </c>
       <c r="D26" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>392</v>
+        <v>424</v>
       </c>
       <c r="E26" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1761</v>
+        <v>1726</v>
       </c>
       <c r="F26" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46269</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -1103,19 +1103,19 @@
       </c>
       <c r="C27" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>967</v>
+        <v>1636</v>
       </c>
       <c r="D27" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>308</v>
+        <v>1569</v>
       </c>
       <c r="E27" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>630</v>
+        <v>2411</v>
       </c>
       <c r="F27" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46023</v>
+        <v>46101</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -1127,19 +1127,19 @@
       </c>
       <c r="C28" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1488</v>
+        <v>690</v>
       </c>
       <c r="D28" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>973</v>
+        <v>212</v>
       </c>
       <c r="E28" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2240</v>
+        <v>475</v>
       </c>
       <c r="F28" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46190</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -1151,19 +1151,19 @@
       </c>
       <c r="C29" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2370</v>
+        <v>651</v>
       </c>
       <c r="D29" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>274</v>
+        <v>1029</v>
       </c>
       <c r="E29" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1061</v>
+        <v>1042</v>
       </c>
       <c r="F29" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46063</v>
+        <v>46059</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -1175,19 +1175,19 @@
       </c>
       <c r="C30" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>150</v>
+        <v>261</v>
       </c>
       <c r="D30" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1190</v>
+        <v>148</v>
       </c>
       <c r="E30" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1912</v>
+        <v>1000</v>
       </c>
       <c r="F30" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46283</v>
+        <v>46285</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -1199,19 +1199,19 @@
       </c>
       <c r="C31" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>370</v>
+        <v>735</v>
       </c>
       <c r="D31" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1458</v>
+        <v>273</v>
       </c>
       <c r="E31" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2399</v>
+        <v>477</v>
       </c>
       <c r="F31" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46066</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
@@ -1223,19 +1223,19 @@
       </c>
       <c r="C32" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1234</v>
+        <v>1305</v>
       </c>
       <c r="D32" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>160</v>
+        <v>101</v>
       </c>
       <c r="E32" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1156</v>
+        <v>961</v>
       </c>
       <c r="F32" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46365</v>
+        <v>46324</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
@@ -1247,19 +1247,19 @@
       </c>
       <c r="C33" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1865</v>
+        <v>2225</v>
       </c>
       <c r="D33" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>346</v>
+        <v>241</v>
       </c>
       <c r="E33" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>400</v>
+        <v>387</v>
       </c>
       <c r="F33" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46114</v>
+        <v>46056</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -1271,19 +1271,19 @@
       </c>
       <c r="C34" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1786</v>
+        <v>1255</v>
       </c>
       <c r="D34" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>460</v>
+        <v>1023</v>
       </c>
       <c r="E34" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1429</v>
+        <v>1693</v>
       </c>
       <c r="F34" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46035</v>
+        <v>46056</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
@@ -1295,19 +1295,19 @@
       </c>
       <c r="C35" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>315</v>
+        <v>1496</v>
       </c>
       <c r="D35" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>156</v>
+        <v>350</v>
       </c>
       <c r="E35" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>254</v>
+        <v>1540</v>
       </c>
       <c r="F35" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46387</v>
+        <v>46057</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
@@ -1319,19 +1319,19 @@
       </c>
       <c r="C36" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>554</v>
+        <v>878</v>
       </c>
       <c r="D36" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>713</v>
+        <v>304</v>
       </c>
       <c r="E36" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1562</v>
+        <v>670</v>
       </c>
       <c r="F36" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46274</v>
+        <v>46137</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -1343,19 +1343,19 @@
       </c>
       <c r="C37" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1383</v>
+        <v>1178</v>
       </c>
       <c r="D37" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1754</v>
+        <v>1708</v>
       </c>
       <c r="E37" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2152</v>
+        <v>2365</v>
       </c>
       <c r="F37" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46046</v>
+        <v>46053</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -1367,19 +1367,19 @@
       </c>
       <c r="C38" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>665</v>
+        <v>2357</v>
       </c>
       <c r="D38" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>468</v>
+        <v>303</v>
       </c>
       <c r="E38" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>576</v>
+        <v>757</v>
       </c>
       <c r="F38" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46064</v>
+        <v>46135</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -1391,19 +1391,19 @@
       </c>
       <c r="C39" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>165</v>
+        <v>254</v>
       </c>
       <c r="D39" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>383</v>
+        <v>731</v>
       </c>
       <c r="E39" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1364</v>
+        <v>1081</v>
       </c>
       <c r="F39" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46083</v>
+        <v>46085</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -1415,19 +1415,19 @@
       </c>
       <c r="C40" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1610</v>
+        <v>1958</v>
       </c>
       <c r="D40" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>239</v>
+        <v>840</v>
       </c>
       <c r="E40" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2328</v>
+        <v>1439</v>
       </c>
       <c r="F40" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46269</v>
+        <v>46291</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -1439,19 +1439,19 @@
       </c>
       <c r="C41" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>341</v>
+        <v>938</v>
       </c>
       <c r="D41" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>243</v>
+        <v>550</v>
       </c>
       <c r="E41" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>261</v>
+        <v>1689</v>
       </c>
       <c r="F41" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46181</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -1463,19 +1463,19 @@
       </c>
       <c r="C42" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1437</v>
+        <v>1586</v>
       </c>
       <c r="D42" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>404</v>
+        <v>1010</v>
       </c>
       <c r="E42" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>955</v>
+        <v>1359</v>
       </c>
       <c r="F42" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46288</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1487,19 +1487,19 @@
       </c>
       <c r="C43" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1260</v>
+        <v>1195</v>
       </c>
       <c r="D43" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>754</v>
+        <v>1409</v>
       </c>
       <c r="E43" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1208</v>
+        <v>2340</v>
       </c>
       <c r="F43" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46384</v>
+        <v>46086</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -1511,19 +1511,19 @@
       </c>
       <c r="C44" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1408</v>
+        <v>2406</v>
       </c>
       <c r="D44" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>638</v>
+        <v>298</v>
       </c>
       <c r="E44" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>866</v>
+        <v>897</v>
       </c>
       <c r="F44" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46163</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -1535,19 +1535,19 @@
       </c>
       <c r="C45" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1166</v>
+        <v>2261</v>
       </c>
       <c r="D45" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>207</v>
+        <v>1688</v>
       </c>
       <c r="E45" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>223</v>
+        <v>1782</v>
       </c>
       <c r="F45" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46145</v>
+        <v>46068</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1559,19 +1559,19 @@
       </c>
       <c r="C46" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2095</v>
+        <v>695</v>
       </c>
       <c r="D46" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>568</v>
+        <v>1159</v>
       </c>
       <c r="E46" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>652</v>
+        <v>1818</v>
       </c>
       <c r="F46" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46303</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -1583,19 +1583,19 @@
       </c>
       <c r="C47" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>910</v>
+        <v>625</v>
       </c>
       <c r="D47" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>315</v>
+        <v>939</v>
       </c>
       <c r="E47" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>578</v>
+        <v>2254</v>
       </c>
       <c r="F47" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46024</v>
+        <v>46372</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -1607,19 +1607,19 @@
       </c>
       <c r="C48" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>707</v>
+        <v>913</v>
       </c>
       <c r="D48" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>116</v>
+        <v>205</v>
       </c>
       <c r="E48" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>149</v>
+        <v>902</v>
       </c>
       <c r="F48" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46208</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -1631,19 +1631,19 @@
       </c>
       <c r="C49" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>1597</v>
+        <v>2029</v>
       </c>
       <c r="D49" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1466</v>
+        <v>112</v>
       </c>
       <c r="E49" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2254</v>
+        <v>565</v>
       </c>
       <c r="F49" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46234</v>
+        <v>46263</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -1655,19 +1655,19 @@
       </c>
       <c r="C50" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2448</v>
+        <v>1247</v>
       </c>
       <c r="D50" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1078</v>
+        <v>1428</v>
       </c>
       <c r="E50" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>2323</v>
+        <v>2228</v>
       </c>
       <c r="F50" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46243</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -1679,19 +1679,19 @@
       </c>
       <c r="C51" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>2234</v>
+        <v>1615</v>
       </c>
       <c r="D51" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>1069</v>
+        <v>898</v>
       </c>
       <c r="E51" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1155</v>
+        <v>1893</v>
       </c>
       <c r="F51" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46193</v>
+        <v>46335</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -1703,19 +1703,19 @@
       </c>
       <c r="C52" s="1">
         <f t="shared" ca="1" si="2"/>
-        <v>151</v>
+        <v>536</v>
       </c>
       <c r="D52" s="1">
         <f t="shared" ca="1" si="3"/>
-        <v>708</v>
+        <v>1920</v>
       </c>
       <c r="E52" s="1">
         <f t="shared" ca="1" si="4"/>
-        <v>1111</v>
+        <v>2003</v>
       </c>
       <c r="F52" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46336</v>
+        <v>46370</v>
       </c>
     </row>
   </sheetData>

</xml_diff>